<commit_message>
test commit Soniya token
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_NSV_TRADSL_TAX.xlsx
+++ b/SuppXLS/Scen_NSV_TRADSL_TAX.xlsx
@@ -51,27 +51,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>~TFM_INS</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>REG1</t>
+  </si>
   <si>
     <t>Cset_CN</t>
   </si>
   <si>
-    <t>TRADSL</t>
-  </si>
-  <si>
-    <t>Pset_PN</t>
+    <t>TC*</t>
   </si>
   <si>
     <t>REG2</t>
   </si>
   <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>~TFM_INS</t>
-  </si>
-  <si>
-    <t>REG1</t>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>Trans - Insert</t>
+  </si>
+  <si>
+    <t>TimeSlice</t>
   </si>
   <si>
     <t>FLO_TAX</t>
@@ -81,19 +90,13 @@
 </t>
   </si>
   <si>
-    <t>TC*</t>
-  </si>
-  <si>
-    <t>TimeSlice</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Trans - Insert</t>
+    <t>Pset_PN</t>
+  </si>
+  <si>
+    <t>TRADSL</t>
+  </si>
+  <si>
+    <t>yjhbj</t>
   </si>
 </sst>
 </file>
@@ -849,48 +852,48 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="2:9" ht="15">
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="2:13" ht="15.75" thickBot="1">
       <c r="B3" s="10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="M3" s="8" t="s">
         <v>11</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="M3" s="8" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="4" spans="4:12" ht="15">
       <c r="D4" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E4" s="7">
         <v>2015</v>
@@ -902,21 +905,21 @@
         <v>10</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="4:11" ht="15">
       <c r="D5" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E5" s="7">
         <v>2050</v>
@@ -928,18 +931,18 @@
         <v>20</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="4:13" ht="15">
       <c r="D6" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E6" s="7">
         <v>0</v>
@@ -951,13 +954,13 @@
         <v>5</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test commit for token testing
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_NSV_TRADSL_TAX.xlsx
+++ b/SuppXLS/Scen_NSV_TRADSL_TAX.xlsx
@@ -51,52 +51,49 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
-  <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>~TFM_INS</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>REG1</t>
-  </si>
-  <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>TC*</t>
-  </si>
-  <si>
-    <t>REG2</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
-    <t>Trans - Insert</t>
-  </si>
-  <si>
-    <t>TimeSlice</t>
-  </si>
-  <si>
-    <t>FLO_TAX</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
   <si>
     <t xml:space="preserve">
 </t>
   </si>
   <si>
+    <t>TRADSL</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
+  </si>
+  <si>
     <t>Pset_PN</t>
   </si>
   <si>
-    <t>TRADSL</t>
-  </si>
-  <si>
-    <t>yjhbj</t>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>TimeSlice</t>
+  </si>
+  <si>
+    <t>REG2</t>
+  </si>
+  <si>
+    <t>FLO_TAX</t>
+  </si>
+  <si>
+    <t>TC*</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>REG1</t>
+  </si>
+  <si>
+    <t>~TFM_INS</t>
+  </si>
+  <si>
+    <t>Trans - Insert</t>
   </si>
 </sst>
 </file>
@@ -251,7 +248,7 @@
       <protection/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -286,6 +283,10 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
       <protection/>
     </xf>
   </cellXfs>
@@ -852,48 +853,48 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="2:9" ht="15">
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="2:13" ht="15.75" thickBot="1">
       <c r="B3" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>7</v>
-      </c>
       <c r="D3" s="10" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G3" s="11" t="s">
         <v>6</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="4:12" ht="15">
       <c r="D4" s="6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E4" s="7">
         <v>2015</v>
@@ -905,21 +906,21 @@
         <v>10</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="4:11" ht="15">
       <c r="D5" s="6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E5" s="7">
         <v>2050</v>
@@ -931,18 +932,18 @@
         <v>20</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="4:13" ht="15">
       <c r="D6" s="6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E6" s="7">
         <v>0</v>
@@ -954,13 +955,13 @@
         <v>5</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="M6" s="9" t="s">
-        <v>14</v>
+        <v>1</v>
+      </c>
+      <c r="M6" s="13" t="s">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
testing commit test commit use name
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_NSV_TRADSL_TAX.xlsx
+++ b/SuppXLS/Scen_NSV_TRADSL_TAX.xlsx
@@ -51,33 +51,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="15">
-  <si>
-    <t>Trans - Insert</t>
-  </si>
-  <si>
-    <t>~TFM_INS</t>
-  </si>
-  <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Pset_PN</t>
-  </si>
-  <si>
-    <t>FLO_TAX</t>
-  </si>
-  <si>
-    <t>REG1</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
-    <t>TimeSlice</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="14">
+  <si>
+    <t>TRADSL</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -87,16 +63,37 @@
     <t>Cset_CN</t>
   </si>
   <si>
+    <t>REG1</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>Pset_PN</t>
+  </si>
+  <si>
+    <t>FLO_TAX</t>
+  </si>
+  <si>
+    <t>TC*</t>
+  </si>
+  <si>
+    <t>Trans - Insert</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
     <t>REG2</t>
   </si>
   <si>
-    <t>TC*</t>
-  </si>
-  <si>
-    <t>TRADSL</t>
-  </si>
-  <si>
-    <t>adeads</t>
+    <t>TimeSlice</t>
+  </si>
+  <si>
+    <t>~TFM_INS</t>
+  </si>
+  <si>
+    <t>Attribute</t>
   </si>
 </sst>
 </file>
@@ -856,48 +853,48 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="2:9" ht="15">
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="2:13" ht="15.75" thickBot="1">
       <c r="B3" s="10" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>10</v>
-      </c>
       <c r="M3" s="8" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="4:12" ht="15">
       <c r="D4" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4" s="7">
         <v>2015</v>
@@ -909,21 +906,21 @@
         <v>10</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="4:12" ht="15">
       <c r="D5" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" s="7">
         <v>2050</v>
@@ -935,21 +932,21 @@
         <v>20</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="L5" t="s">
-        <v>14</v>
+        <v>1</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="4:13" ht="15">
       <c r="D6" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" s="7">
         <v>0</v>
@@ -961,13 +958,13 @@
         <v>5</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="M6" s="13" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test push for Veda Online
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_NSV_TRADSL_TAX.xlsx
+++ b/SuppXLS/Scen_NSV_TRADSL_TAX.xlsx
@@ -51,49 +51,52 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="15">
+  <si>
+    <t>~TFM_INS</t>
+  </si>
+  <si>
+    <t>Trans - Insert</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>REG2</t>
+  </si>
+  <si>
+    <t>hjkj</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>TimeSlice</t>
+  </si>
   <si>
     <t>TRADSL</t>
+  </si>
+  <si>
+    <t>Pset_PN</t>
+  </si>
+  <si>
+    <t>REG1</t>
+  </si>
+  <si>
+    <t>FLO_TAX</t>
+  </si>
+  <si>
+    <t>TC*</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
   </si>
   <si>
     <t xml:space="preserve">
 </t>
-  </si>
-  <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>REG1</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
-    <t>Pset_PN</t>
-  </si>
-  <si>
-    <t>FLO_TAX</t>
-  </si>
-  <si>
-    <t>TC*</t>
-  </si>
-  <si>
-    <t>Trans - Insert</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>REG2</t>
-  </si>
-  <si>
-    <t>TimeSlice</t>
-  </si>
-  <si>
-    <t>~TFM_INS</t>
-  </si>
-  <si>
-    <t>Attribute</t>
   </si>
 </sst>
 </file>
@@ -853,48 +856,48 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="2:9" ht="15">
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="2:13" ht="15.75" thickBot="1">
       <c r="B3" s="10" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="M3" s="8" t="s">
         <v>4</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="M3" s="8" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="4" spans="4:12" ht="15">
       <c r="D4" s="6" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E4" s="7">
         <v>2015</v>
@@ -906,21 +909,21 @@
         <v>10</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="4:12" ht="15">
       <c r="D5" s="6" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E5" s="7">
         <v>2050</v>
@@ -932,21 +935,21 @@
         <v>20</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="4:13" ht="15">
       <c r="D6" s="6" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E6" s="7">
         <v>0</v>
@@ -958,13 +961,13 @@
         <v>5</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M6" s="13" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>